<commit_message>
Chore: Correction to database design
</commit_message>
<xml_diff>
--- a/02-Design/database-normalization/Normalización SECSS.xlsx
+++ b/02-Design/database-normalization/Normalización SECSS.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/BC664D82486B06FA/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve\OneDrive\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="358" documentId="8_{62C522AD-2817-4FCE-8437-BDB93046B38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E545F7C9-9CA5-45E1-AF1E-C0A1DF6A2730}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF2F189-8142-48E6-AD67-FA07D05B3B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9DE7D6E0-6F9A-487E-9F24-0C1E12FA1321}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="SECSS" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="163">
   <si>
     <t>id</t>
   </si>
@@ -368,12 +368,6 @@
     <t>VEHICULO INVITADO</t>
   </si>
   <si>
-    <t>hora_entrada</t>
-  </si>
-  <si>
-    <t>hora_salida</t>
-  </si>
-  <si>
     <t>id_perfil_celador</t>
   </si>
   <si>
@@ -504,16 +498,49 @@
   </si>
   <si>
     <t>Ya cambiamos tus datos a…</t>
+  </si>
+  <si>
+    <t>nombre_centro</t>
+  </si>
+  <si>
+    <t>CEET</t>
+  </si>
+  <si>
+    <t>CENTRO</t>
+  </si>
+  <si>
+    <t>id_centro</t>
+  </si>
+  <si>
+    <t>imagen_url_identificacion_vehiculo</t>
+  </si>
+  <si>
+    <t>imagen_url_vehiculo</t>
+  </si>
+  <si>
+    <t>tipo_ingreso</t>
+  </si>
+  <si>
+    <t>ENTRADA</t>
+  </si>
+  <si>
+    <t>SALIDA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -539,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -557,11 +584,61 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="111">
+  <dxfs count="118">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="d/mm/yyyy\ h:mm"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -655,10 +732,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="d/mm/yyyy\ h:mm"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -694,30 +767,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="d/mm/yyyy"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -931,10 +980,10 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Estilo de tabla 1" pivot="0" count="4" xr9:uid="{FFE869F8-77F0-44C9-8F34-976B4A70E0D5}">
-      <tableStyleElement type="wholeTable" dxfId="110"/>
-      <tableStyleElement type="headerRow" dxfId="109"/>
-      <tableStyleElement type="firstRowStripe" dxfId="108"/>
-      <tableStyleElement type="secondRowStripe" dxfId="107"/>
+      <tableStyleElement type="wholeTable" dxfId="117"/>
+      <tableStyleElement type="headerRow" dxfId="116"/>
+      <tableStyleElement type="firstRowStripe" dxfId="115"/>
+      <tableStyleElement type="secondRowStripe" dxfId="114"/>
     </tableStyle>
     <tableStyle name="Estilo de tabla 2" pivot="0" count="0" xr9:uid="{CF3F03A1-9E19-4720-96D7-711A5CA0D05F}"/>
   </tableStyles>
@@ -949,128 +998,128 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1E27DE7D-6377-4FED-8629-F5BDD9D7FB4E}" name="Tabla6" displayName="Tabla6" ref="C4:D9" totalsRowShown="0" dataDxfId="106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1E27DE7D-6377-4FED-8629-F5BDD9D7FB4E}" name="Tabla6" displayName="Tabla6" ref="C4:D9" totalsRowShown="0" dataDxfId="113">
   <autoFilter ref="C4:D9" xr:uid="{1E27DE7D-6377-4FED-8629-F5BDD9D7FB4E}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C8805EA9-577E-48FD-B540-C43FCC337A75}" name="id" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{DD226C46-6BFF-4EA0-9379-F8EEADEAD146}" name="rol" dataDxfId="104"/>
+    <tableColumn id="1" xr3:uid="{C8805EA9-577E-48FD-B540-C43FCC337A75}" name="id" dataDxfId="112"/>
+    <tableColumn id="2" xr3:uid="{DD226C46-6BFF-4EA0-9379-F8EEADEAD146}" name="rol" dataDxfId="111"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3CBD9C2-7EB8-4AF8-9C36-8559156141D8}" name="Tabla5" displayName="Tabla5" ref="U4:Y7" totalsRowShown="0" dataDxfId="68">
-  <autoFilter ref="U4:Y7" xr:uid="{E3CBD9C2-7EB8-4AF8-9C36-8559156141D8}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{EEA0E70A-3052-4D25-ADD6-531EAEFD31E1}" name="id" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{4AC020D0-0054-4F10-9748-D42DEB35E95E}" name="id_tipo_vehiculo" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{76D7BB69-740C-4176-AF68-52662BCAD3D0}" name="marca" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{E35E5783-7D86-48E3-91A2-D1EDDF158B42}" name="color" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{885DF92E-D802-4D0A-9050-445984D55BA3}" name="imagen_url_targeta_propiedad" dataDxfId="63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3CBD9C2-7EB8-4AF8-9C36-8559156141D8}" name="Tabla5" displayName="Tabla5" ref="U4:AA7" totalsRowShown="0" dataDxfId="83">
+  <autoFilter ref="U4:AA7" xr:uid="{E3CBD9C2-7EB8-4AF8-9C36-8559156141D8}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{EEA0E70A-3052-4D25-ADD6-531EAEFD31E1}" name="id" dataDxfId="82"/>
+    <tableColumn id="2" xr3:uid="{4AC020D0-0054-4F10-9748-D42DEB35E95E}" name="id_tipo_vehiculo" dataDxfId="81"/>
+    <tableColumn id="3" xr3:uid="{76D7BB69-740C-4176-AF68-52662BCAD3D0}" name="marca" dataDxfId="80"/>
+    <tableColumn id="4" xr3:uid="{E35E5783-7D86-48E3-91A2-D1EDDF158B42}" name="color" dataDxfId="79"/>
+    <tableColumn id="5" xr3:uid="{885DF92E-D802-4D0A-9050-445984D55BA3}" name="imagen_url_targeta_propiedad" dataDxfId="78"/>
+    <tableColumn id="6" xr3:uid="{0EE9B581-482E-4759-ACF1-E724CA278F9E}" name="imagen_url_identificacion_vehiculo" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{E4A99698-CB0C-454D-8B4A-5DDA8F0EDCDC}" name="imagen_url_vehiculo" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{89F0F7A4-13AE-49C1-9BFB-759D0FFFA1C7}" name="Tabla12" displayName="Tabla12" ref="U17:AA19" totalsRowShown="0" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{89F0F7A4-13AE-49C1-9BFB-759D0FFFA1C7}" name="Tabla12" displayName="Tabla12" ref="U17:AA19" totalsRowShown="0" dataDxfId="77">
   <autoFilter ref="U17:AA19" xr:uid="{89F0F7A4-13AE-49C1-9BFB-759D0FFFA1C7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{BB9E9419-3D08-4785-963C-AAFB08010CB5}" name="id" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{7E27379E-B0FA-45CF-BA46-AED1B55BEE48}" name="id_vehiculo" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{6F45A3ED-55E0-401A-8D9C-426CB36A0CE2}" name="placa" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{C23C9BDC-AB7F-4FFC-85B8-90D7232ED94E}" name="cilindraje" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{3A4A1D19-8B51-4E8E-B045-046E92BC3791}" name="modelo" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{9474396C-5478-4824-B8E1-51D739875400}" name="imagen_url_soat" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{8497878E-4856-47BD-8C88-E8EE9023604C}" name="imagen_url_tecnomecanica" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{BB9E9419-3D08-4785-963C-AAFB08010CB5}" name="id" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{7E27379E-B0FA-45CF-BA46-AED1B55BEE48}" name="id_vehiculo" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{6F45A3ED-55E0-401A-8D9C-426CB36A0CE2}" name="placa" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{C23C9BDC-AB7F-4FFC-85B8-90D7232ED94E}" name="cilindraje" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{3A4A1D19-8B51-4E8E-B045-046E92BC3791}" name="modelo" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{9474396C-5478-4824-B8E1-51D739875400}" name="imagen_url_soat" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{8497878E-4856-47BD-8C88-E8EE9023604C}" name="imagen_url_tecnomecanica" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{7FBFFF43-7DAF-4B6F-9D32-F3850F11F95A}" name="Tabla13" displayName="Tabla13" ref="U23:X24" totalsRowShown="0" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{7FBFFF43-7DAF-4B6F-9D32-F3850F11F95A}" name="Tabla13" displayName="Tabla13" ref="U23:X24" totalsRowShown="0" dataDxfId="69">
   <autoFilter ref="U23:X24" xr:uid="{7FBFFF43-7DAF-4B6F-9D32-F3850F11F95A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E5C0780E-225C-4682-997C-AB969AEB218C}" name="id" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{058A41F2-EC3D-48AF-A063-FDFB082FE7DC}" name="id_vehiculo" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{25C1ABDB-01FC-4190-AA07-27D42AF54B3A}" name="numero_marco" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{38A62538-BFB4-469D-939C-CD8A45E875EF}" name="clase_bicicleta" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{E5C0780E-225C-4682-997C-AB969AEB218C}" name="id" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{058A41F2-EC3D-48AF-A063-FDFB082FE7DC}" name="id_vehiculo" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{25C1ABDB-01FC-4190-AA07-27D42AF54B3A}" name="numero_marco" dataDxfId="66"/>
+    <tableColumn id="4" xr3:uid="{38A62538-BFB4-469D-939C-CD8A45E875EF}" name="clase_bicicleta" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{C8A325AF-20E8-4D7D-915D-163F12721056}" name="Tabla14" displayName="Tabla14" ref="U11:V13" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{C8A325AF-20E8-4D7D-915D-163F12721056}" name="Tabla14" displayName="Tabla14" ref="U11:V13" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
   <autoFilter ref="U11:V13" xr:uid="{C8A325AF-20E8-4D7D-915D-163F12721056}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{5DC0074D-2812-4EF8-BAA7-4D6B6EF69BBA}" name="id" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{BE483DB7-FB67-4A94-A556-0E1FBDEDA310}" name="nombre_vehiculo" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{5DC0074D-2812-4EF8-BAA7-4D6B6EF69BBA}" name="id" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{BE483DB7-FB67-4A94-A556-0E1FBDEDA310}" name="nombre_vehiculo" dataDxfId="61"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{5A808533-7F6C-46E2-A454-A4512BE81AC7}" name="Tabla15" displayName="Tabla15" ref="U28:Z30" totalsRowShown="0" dataDxfId="45">
-  <autoFilter ref="U28:Z30" xr:uid="{5A808533-7F6C-46E2-A454-A4512BE81AC7}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{568AB0A3-C028-4AA8-BA21-8C7BB0B75261}" name="id_aprendiz" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{577A6B5D-5111-44FE-850E-BBE7E867F5C3}" name="id_vehiculo" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{943234B9-0035-4A73-B149-D21D56120637}" name="fecha_vinculacion" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{F8DF713C-DAD3-48F5-962C-96D3C5BCE65D}" name="fecha_terminacion" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{E161AD1C-3616-46B5-BE9D-96E027F2F299}" name="estado" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{CD114081-A840-4516-AAF7-F9B8F9A1DE67}" name="id_administrador" dataDxfId="39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{5A808533-7F6C-46E2-A454-A4512BE81AC7}" name="Tabla15" displayName="Tabla15" ref="U28:AB30" totalsRowShown="0" dataDxfId="60">
+  <autoFilter ref="U28:AB30" xr:uid="{5A808533-7F6C-46E2-A454-A4512BE81AC7}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{568AB0A3-C028-4AA8-BA21-8C7BB0B75261}" name="id_aprendiz" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{577A6B5D-5111-44FE-850E-BBE7E867F5C3}" name="id_vehiculo" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{943234B9-0035-4A73-B149-D21D56120637}" name="fecha_vinculacion" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{F8DF713C-DAD3-48F5-962C-96D3C5BCE65D}" name="fecha_terminacion" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{E161AD1C-3616-46B5-BE9D-96E027F2F299}" name="estado" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{CD114081-A840-4516-AAF7-F9B8F9A1DE67}" name="id_administrador" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{9422B8A0-1A10-4B16-BEC8-0446422DF7F4}" name="imagen_url_carnet_sena" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{A50B0A27-A630-4312-9270-CFE2D574A5AC}" name="id_centro" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{5F27C29D-FBF0-4C04-8C41-2F1C4E6828F1}" name="Tabla17" displayName="Tabla17" ref="U34:V35" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{5F27C29D-FBF0-4C04-8C41-2F1C4E6828F1}" name="Tabla17" displayName="Tabla17" ref="U34:V35" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="U34:V35" xr:uid="{5F27C29D-FBF0-4C04-8C41-2F1C4E6828F1}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{CCFBDAE3-387F-4F47-8336-5D2E34250FEB}" name="id_usuario" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{9135BFE3-50AE-4078-81F0-72550C4931E1}" name="id_vehiculo" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{CCFBDAE3-387F-4F47-8336-5D2E34250FEB}" name="id_usuario" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{9135BFE3-50AE-4078-81F0-72550C4931E1}" name="id_vehiculo" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{A9B537D7-9686-48F9-9881-A9E607B1141F}" name="Tabla16" displayName="Tabla16" ref="U39:AA40" totalsRowShown="0" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{A9B537D7-9686-48F9-9881-A9E607B1141F}" name="Tabla16" displayName="Tabla16" ref="U39:AA40" totalsRowShown="0" dataDxfId="49">
   <autoFilter ref="U39:AA40" xr:uid="{A9B537D7-9686-48F9-9881-A9E607B1141F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{627F89AC-CCE3-48ED-A5E8-95D4F1D70B2F}" name="id" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{3B979D23-C57E-4219-A061-6FF3089EFE9F}" name="id_aprendiz" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{3DD18A48-9099-4DAA-923D-2ACB59DAFC11}" name="id_vehiculo" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{83B3E2BA-A8B3-433B-8DF8-9267F7C19D42}" name="hora_entrada" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{AC076088-A54B-482E-8D85-2CE7A00C70EC}" name="hora_salida" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{1A1E8AA3-4EBC-4C13-862D-E493B6E28B2B}" name="id_perfil_celador" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{9289EFF8-8298-49E7-9008-23631765F89C}" name="estado" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{627F89AC-CCE3-48ED-A5E8-95D4F1D70B2F}" name="id" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{3B979D23-C57E-4219-A061-6FF3089EFE9F}" name="id_aprendiz" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{3DD18A48-9099-4DAA-923D-2ACB59DAFC11}" name="id_vehiculo" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{83B3E2BA-A8B3-433B-8DF8-9267F7C19D42}" name="fecha_hora" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{AC076088-A54B-482E-8D85-2CE7A00C70EC}" name="id_perfil_celador" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{1A1E8AA3-4EBC-4C13-862D-E493B6E28B2B}" name="tipo_ingreso" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{9289EFF8-8298-49E7-9008-23631765F89C}" name="estado" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{437C5D5A-01DB-4D45-BF18-35FC22C1874F}" name="Tabla19" displayName="Tabla19" ref="U44:AA45" totalsRowShown="0" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{437C5D5A-01DB-4D45-BF18-35FC22C1874F}" name="Tabla19" displayName="Tabla19" ref="U44:AA45" totalsRowShown="0" dataDxfId="42">
   <autoFilter ref="U44:AA45" xr:uid="{437C5D5A-01DB-4D45-BF18-35FC22C1874F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{622F7CED-2DD9-4C33-A18F-4E9BBA1AE116}" name="id" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{AFB15B71-B49B-4895-877A-7CD80CC519E4}" name="id_usuario" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{6D885132-95FD-4ADD-8C0D-BE06641C307A}" name="id_vehiculo" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{AA3AD6DF-C556-4BFA-9BF5-1DA1DD1CD268}" name="hora_entrada" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{C600F355-11E1-4436-AF7E-A4B7D628927F}" name="hora_salida" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{B042C918-8542-47CD-BE7C-BFBE32702A2E}" name="id_perfil_celador" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{3F08BBAE-33DD-4D74-AB41-65F243CC97B1}" name="estado" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{622F7CED-2DD9-4C33-A18F-4E9BBA1AE116}" name="id" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{AFB15B71-B49B-4895-877A-7CD80CC519E4}" name="id_usuario" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{6D885132-95FD-4ADD-8C0D-BE06641C307A}" name="id_vehiculo" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{AA3AD6DF-C556-4BFA-9BF5-1DA1DD1CD268}" name="fecha_hora" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{C600F355-11E1-4436-AF7E-A4B7D628927F}" name="id_perfil_celador" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{B042C918-8542-47CD-BE7C-BFBE32702A2E}" name="tipo_ingreso" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{3F08BBAE-33DD-4D74-AB41-65F243CC97B1}" name="estado" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1083,7 +1132,7 @@
     <tableColumn id="1" xr3:uid="{F76C113A-5C2C-430F-9017-54D71D0FD0BF}" name="id"/>
     <tableColumn id="2" xr3:uid="{65DDB87A-B754-4761-BAE3-C46B7D24688B}" name="id_tipo_reporte"/>
     <tableColumn id="3" xr3:uid="{8881179A-9C47-46CE-ADCD-582036DED36A}" name="id_perfil_celador"/>
-    <tableColumn id="4" xr3:uid="{C48DBBE6-03BF-40AF-8D15-B39D8A03B665}" name="fecha_hora" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{C48DBBE6-03BF-40AF-8D15-B39D8A03B665}" name="fecha_hora" dataDxfId="34"/>
     <tableColumn id="5" xr3:uid="{D39D4E99-72C6-4277-8AB9-CDC4D38554CE}" name="asunto"/>
     <tableColumn id="6" xr3:uid="{58297757-433C-4520-AE83-9916AE34FDA0}" name="cuerpo"/>
     <tableColumn id="7" xr3:uid="{38B33E21-5A6D-4B55-B4CF-0BB6EFC7C998}" name="estado"/>
@@ -1093,23 +1142,23 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{FE8FA8ED-4E96-4E53-BE08-B27AC6E1EA3B}" name="Tabla18" displayName="Tabla18" ref="O30:P33" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{FE8FA8ED-4E96-4E53-BE08-B27AC6E1EA3B}" name="Tabla18" displayName="Tabla18" ref="O30:P33" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="O30:P33" xr:uid="{FE8FA8ED-4E96-4E53-BE08-B27AC6E1EA3B}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A1096C5F-FCE7-4DE8-B491-2BDE248B1637}" name="id" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{674A617F-65F1-4AEC-A4D2-E84BC65912CE}" name="nombre_reporte" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{A1096C5F-FCE7-4DE8-B491-2BDE248B1637}" name="id" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{674A617F-65F1-4AEC-A4D2-E84BC65912CE}" name="nombre_reporte" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{78564E9F-BE6A-4F59-A0D1-CB7752282409}" name="Tabla7" displayName="Tabla7" ref="C13:E19" totalsRowShown="0" dataDxfId="103">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{78564E9F-BE6A-4F59-A0D1-CB7752282409}" name="Tabla7" displayName="Tabla7" ref="C13:E19" totalsRowShown="0" dataDxfId="110">
   <autoFilter ref="C13:E19" xr:uid="{78564E9F-BE6A-4F59-A0D1-CB7752282409}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B8728401-897E-4A6B-8AAA-747B72E37E18}" name="id_cuenta" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{BECA1369-F4ED-48E7-BAED-DAA79C158A35}" name="id_rol" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{7EAAFB1B-C0D6-4293-A95F-A4D2A4A89881}" name="estado" dataDxfId="100"/>
+    <tableColumn id="1" xr3:uid="{B8728401-897E-4A6B-8AAA-747B72E37E18}" name="id_cuenta" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{BECA1369-F4ED-48E7-BAED-DAA79C158A35}" name="id_rol" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{7EAAFB1B-C0D6-4293-A95F-A4D2A4A89881}" name="estado" dataDxfId="107"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1145,7 +1194,7 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{883ACAD4-6A57-46E7-BD3F-503B79F0C0FB}" name="id"/>
     <tableColumn id="2" xr3:uid="{B5C145CD-556F-43C0-8EA6-B7054CF3CF3E}" name="id_usuario"/>
-    <tableColumn id="3" xr3:uid="{65955E4F-FD71-4C8E-9BDE-88A85B6BEE6C}" name="fecha_hora" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{65955E4F-FD71-4C8E-9BDE-88A85B6BEE6C}" name="fecha_hora" dataDxfId="29"/>
     <tableColumn id="4" xr3:uid="{05F189CF-7C3D-4EAC-94E9-960609F5E1F9}" name="asunto"/>
     <tableColumn id="5" xr3:uid="{17120173-9505-4A2E-AF16-2CF4115BCAD9}" name="cuerpo"/>
     <tableColumn id="6" xr3:uid="{A4252E12-2DCA-4D77-8E50-610B9892CC13}" name="estado"/>
@@ -1161,45 +1210,56 @@
     <tableColumn id="1" xr3:uid="{6BEABC92-C379-428B-8FAD-1389B2CE84B2}" name="id"/>
     <tableColumn id="2" xr3:uid="{40F7F64C-CFB5-438A-B5FE-F84C4736A88A}" name="id_pqrs"/>
     <tableColumn id="3" xr3:uid="{E5BD59B6-1B7A-4414-B8CE-98FB0965A2FE}" name="id_administrador"/>
-    <tableColumn id="4" xr3:uid="{9D62A82C-8506-44AB-8376-8D18426338CA}" name="asunto" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{67521C0E-B63B-466D-A575-486A4FD77CB5}" name="cuerpo" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{9D62A82C-8506-44AB-8376-8D18426338CA}" name="asunto" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{67521C0E-B63B-466D-A575-486A4FD77CB5}" name="cuerpo" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{4E041E5B-CBD6-4060-A66B-DB02D8BD0621}" name="Tabla8" displayName="Tabla8" ref="I4:R9" totalsRowShown="0" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{4E041E5B-CBD6-4060-A66B-DB02D8BD0621}" name="Tabla8" displayName="Tabla8" ref="I4:R9" totalsRowShown="0" dataDxfId="26">
   <autoFilter ref="I4:R9" xr:uid="{4E041E5B-CBD6-4060-A66B-DB02D8BD0621}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{ECE1D02E-4052-45D6-BC6A-77B7C67B8BBF}" name="id" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{2A177229-AE89-42E2-93EF-11E78F2A8DB4}" name="correo" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{F8631C45-C80F-4C79-866E-0CB34BE7E0EC}" name="contraseña" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{1F33AB31-18A6-4183-BF07-BF8AAE640235}" name="login" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{9481F810-DE00-489D-B324-A4C7397B9C8B}" name="activated" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{B6A63B95-736E-403D-98F5-08647DB6932D}" name="lang_key" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{88EBAC19-67EF-4789-BB4F-C42B854BEEE4}" name="image_url" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{FDC69377-59A4-43B3-93A1-3D28A3ADA2E5}" name="activation_key" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{86C59CC3-9BE7-487B-ADA1-D2E684F490D7}" name="reset_key" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{2180AD58-4FDF-4A62-AF2A-580C580231BC}" name="reset_date" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{ECE1D02E-4052-45D6-BC6A-77B7C67B8BBF}" name="id" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{2A177229-AE89-42E2-93EF-11E78F2A8DB4}" name="correo" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{F8631C45-C80F-4C79-866E-0CB34BE7E0EC}" name="contraseña" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{1F33AB31-18A6-4183-BF07-BF8AAE640235}" name="login" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{9481F810-DE00-489D-B324-A4C7397B9C8B}" name="activated" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{B6A63B95-736E-403D-98F5-08647DB6932D}" name="lang_key" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{88EBAC19-67EF-4789-BB4F-C42B854BEEE4}" name="image_url" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{FDC69377-59A4-43B3-93A1-3D28A3ADA2E5}" name="activation_key" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{86C59CC3-9BE7-487B-ADA1-D2E684F490D7}" name="reset_key" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{2180AD58-4FDF-4A62-AF2A-580C580231BC}" name="reset_date" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="Estilo de tabla 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{C5ECDDA5-E168-4771-AEF4-1A591A596460}" name="Tabla25" displayName="Tabla25" ref="X34:Y35" totalsRowShown="0" headerRowDxfId="4" dataDxfId="5">
+  <autoFilter ref="X34:Y35" xr:uid="{C5ECDDA5-E168-4771-AEF4-1A591A596460}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{D2D3CD4D-2854-4D60-90ED-B5955915B99D}" name="id" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{FBEF5F1F-09E8-46A1-8D84-33A51B0CB4ED}" name="nombre_centro" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="Estilo de tabla 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A7C71FCD-CCB1-4F06-BD62-B375D82683B7}" name="Tabla9" displayName="Tabla9" ref="I13:Q18" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A7C71FCD-CCB1-4F06-BD62-B375D82683B7}" name="Tabla9" displayName="Tabla9" ref="I13:Q18" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
   <autoFilter ref="I13:Q18" xr:uid="{A7C71FCD-CCB1-4F06-BD62-B375D82683B7}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5EFA8631-A4FA-4EDC-8439-ADED83B34291}" name="id" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{4D3D1C40-8D22-4222-9E74-47EB870CD43C}" name="id_tipo_documento" dataDxfId="96"/>
-    <tableColumn id="3" xr3:uid="{5EDC81AF-9A1E-45DE-BD32-E6AF830F4AF9}" name="numero_documento" dataDxfId="95"/>
-    <tableColumn id="4" xr3:uid="{C00493F7-EE7E-4B01-9D4E-DA1DAB3E6A8B}" name="primer_nombre" dataDxfId="94"/>
-    <tableColumn id="5" xr3:uid="{5D28DD73-6318-4A52-8942-AA4D0639F606}" name="segundo_nombre" dataDxfId="93"/>
-    <tableColumn id="6" xr3:uid="{6F778901-D389-42EA-97C0-2C98C41A890E}" name="primer_apellido" dataDxfId="92"/>
-    <tableColumn id="7" xr3:uid="{4FF7E3BC-F474-4E8B-90C6-9EE1E8D1731A}" name="segundo_apellido" dataDxfId="91"/>
-    <tableColumn id="8" xr3:uid="{051114E5-E907-4792-9B39-3000949AF489}" name="id_cuenta" dataDxfId="90"/>
-    <tableColumn id="9" xr3:uid="{5CE622A0-7219-40ED-948F-33A37FF6D485}" name="n_celular" dataDxfId="89"/>
+    <tableColumn id="1" xr3:uid="{5EFA8631-A4FA-4EDC-8439-ADED83B34291}" name="id" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{4D3D1C40-8D22-4222-9E74-47EB870CD43C}" name="id_tipo_documento" dataDxfId="103"/>
+    <tableColumn id="3" xr3:uid="{5EDC81AF-9A1E-45DE-BD32-E6AF830F4AF9}" name="numero_documento" dataDxfId="102"/>
+    <tableColumn id="4" xr3:uid="{C00493F7-EE7E-4B01-9D4E-DA1DAB3E6A8B}" name="primer_nombre" dataDxfId="101"/>
+    <tableColumn id="5" xr3:uid="{5D28DD73-6318-4A52-8942-AA4D0639F606}" name="segundo_nombre" dataDxfId="100"/>
+    <tableColumn id="6" xr3:uid="{6F778901-D389-42EA-97C0-2C98C41A890E}" name="primer_apellido" dataDxfId="99"/>
+    <tableColumn id="7" xr3:uid="{4FF7E3BC-F474-4E8B-90C6-9EE1E8D1731A}" name="segundo_apellido" dataDxfId="98"/>
+    <tableColumn id="8" xr3:uid="{051114E5-E907-4792-9B39-3000949AF489}" name="id_cuenta" dataDxfId="97"/>
+    <tableColumn id="9" xr3:uid="{5CE622A0-7219-40ED-948F-33A37FF6D485}" name="n_celular" dataDxfId="96"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1219,60 +1279,59 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{547519E5-199F-4232-8B52-CFCF2279A64D}" name="Tabla1" displayName="Tabla1" ref="I23:O25" totalsRowShown="0" dataDxfId="88">
-  <autoFilter ref="I23:O25" xr:uid="{547519E5-199F-4232-8B52-CFCF2279A64D}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{87A3CEE1-465E-474B-AA51-3C0F6FDFA3B6}" name="id" dataDxfId="87"/>
-    <tableColumn id="2" xr3:uid="{ECE57229-5D82-4E9D-B9E1-018BCDD01C04}" name="id_usuario" dataDxfId="86"/>
-    <tableColumn id="3" xr3:uid="{27AD7BDA-6260-47A1-B066-A6162BF8764C}" name="ficha" dataDxfId="85"/>
-    <tableColumn id="4" xr3:uid="{D31D43E2-69F4-4F3B-AFBC-32C0C0752508}" name="imagen_url_aprendiz" dataDxfId="84"/>
-    <tableColumn id="5" xr3:uid="{6A15507B-8FDB-4987-B8BC-D8F145CC5C93}" name="imagen_url_identificacion" dataDxfId="83"/>
-    <tableColumn id="6" xr3:uid="{760A041E-EE00-4BEB-A283-FF6C9F2C49DD}" name="direccion" dataDxfId="82"/>
-    <tableColumn id="7" xr3:uid="{70E88ADF-ECED-4F13-9C81-63AAEE1666B0}" name="imagen_url_carnet_sena" dataDxfId="81"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{547519E5-199F-4232-8B52-CFCF2279A64D}" name="Tabla1" displayName="Tabla1" ref="I23:N25" totalsRowShown="0" dataDxfId="14">
+  <autoFilter ref="I23:N25" xr:uid="{547519E5-199F-4232-8B52-CFCF2279A64D}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{87A3CEE1-465E-474B-AA51-3C0F6FDFA3B6}" name="id" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{ECE57229-5D82-4E9D-B9E1-018BCDD01C04}" name="id_usuario" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{27AD7BDA-6260-47A1-B066-A6162BF8764C}" name="ficha" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{D31D43E2-69F4-4F3B-AFBC-32C0C0752508}" name="imagen_url_aprendiz" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{6A15507B-8FDB-4987-B8BC-D8F145CC5C93}" name="imagen_url_identificacion" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{760A041E-EE00-4BEB-A283-FF6C9F2C49DD}" name="direccion" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{485F0E44-91D4-44E2-85B1-F48992946F68}" name="Tabla2" displayName="Tabla2" ref="I30:J31" totalsRowShown="0" dataDxfId="80">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{485F0E44-91D4-44E2-85B1-F48992946F68}" name="Tabla2" displayName="Tabla2" ref="I30:J31" totalsRowShown="0" dataDxfId="95">
   <autoFilter ref="I30:J31" xr:uid="{485F0E44-91D4-44E2-85B1-F48992946F68}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{3884A247-87AF-4ADF-9B34-5109E313BC63}" name="id" dataDxfId="79"/>
-    <tableColumn id="2" xr3:uid="{5D87C917-1A49-40F6-B674-42EF74A73219}" name="id_usuario" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{3884A247-87AF-4ADF-9B34-5109E313BC63}" name="id" dataDxfId="94"/>
+    <tableColumn id="2" xr3:uid="{5D87C917-1A49-40F6-B674-42EF74A73219}" name="id_usuario" dataDxfId="93"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA9CB251-F1C2-4D56-BECC-1D8286A19E61}" name="Tabla3" displayName="Tabla3" ref="I35:J36" totalsRowShown="0" dataDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA9CB251-F1C2-4D56-BECC-1D8286A19E61}" name="Tabla3" displayName="Tabla3" ref="I35:J36" totalsRowShown="0" dataDxfId="92">
   <autoFilter ref="I35:J36" xr:uid="{CA9CB251-F1C2-4D56-BECC-1D8286A19E61}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{51FDA44B-A828-4F35-B2CA-A4A4608445A9}" name="id" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{D17B2331-FDFD-4BE5-8174-4CAEB471E364}" name="id_usuario" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{51FDA44B-A828-4F35-B2CA-A4A4608445A9}" name="id" dataDxfId="91"/>
+    <tableColumn id="2" xr3:uid="{D17B2331-FDFD-4BE5-8174-4CAEB471E364}" name="id_usuario" dataDxfId="90"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{A231126D-BBBF-47E1-80CC-5789AE5DAC6A}" name="Tabla11" displayName="Tabla11" ref="L30:M31" totalsRowShown="0" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{A231126D-BBBF-47E1-80CC-5789AE5DAC6A}" name="Tabla11" displayName="Tabla11" ref="L30:M31" totalsRowShown="0" dataDxfId="89">
   <autoFilter ref="L30:M31" xr:uid="{A231126D-BBBF-47E1-80CC-5789AE5DAC6A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{EACDAC2A-51ED-4272-90C4-7AB48F8477E4}" name="id" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{AC563DCF-9B85-4F05-B881-771C007BC0C1}" name="id_usuario" dataDxfId="72"/>
+    <tableColumn id="1" xr3:uid="{EACDAC2A-51ED-4272-90C4-7AB48F8477E4}" name="id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{AC563DCF-9B85-4F05-B881-771C007BC0C1}" name="id_usuario" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BCA383D4-916D-4728-874D-02599B710872}" name="Tabla4" displayName="Tabla4" ref="L35:M36" totalsRowShown="0" dataDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BCA383D4-916D-4728-874D-02599B710872}" name="Tabla4" displayName="Tabla4" ref="L35:M36" totalsRowShown="0" dataDxfId="86">
   <autoFilter ref="L35:M36" xr:uid="{BCA383D4-916D-4728-874D-02599B710872}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E6CEFCF6-3619-4213-B5DB-01DBB1763B2C}" name="id_jefe_seguridad" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{65D23375-8B86-4D55-87F6-429551726BA2}" name="id_celador" dataDxfId="69"/>
+    <tableColumn id="1" xr3:uid="{E6CEFCF6-3619-4213-B5DB-01DBB1763B2C}" name="id_jefe_seguridad" dataDxfId="85"/>
+    <tableColumn id="2" xr3:uid="{65D23375-8B86-4D55-87F6-429551726BA2}" name="id_celador" dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1595,7 +1654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{892F2209-E338-48DD-9DFB-425BF1AF17AC}">
-  <dimension ref="C3:AA60"/>
+  <dimension ref="C3:AB60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
@@ -1617,9 +1676,10 @@
     <col min="23" max="23" width="26.42578125" customWidth="1"/>
     <col min="24" max="24" width="27.7109375" customWidth="1"/>
     <col min="25" max="25" width="43.85546875" customWidth="1"/>
-    <col min="26" max="26" width="27.85546875" customWidth="1"/>
+    <col min="26" max="26" width="34.140625" customWidth="1"/>
     <col min="27" max="27" width="38.7109375" customWidth="1"/>
-    <col min="28" max="29" width="11.5703125" customWidth="1"/>
+    <col min="28" max="28" width="24.140625" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" customWidth="1"/>
     <col min="31" max="31" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1700,6 +1760,12 @@
       <c r="Y4" t="s">
         <v>103</v>
       </c>
+      <c r="Z4" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="5" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C5" s="1">
@@ -1715,7 +1781,7 @@
         <v>21</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L5" s="1">
         <v>1</v>
@@ -1741,7 +1807,13 @@
         <v>78</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="3:27" x14ac:dyDescent="0.25">
@@ -1758,7 +1830,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L6" s="1">
         <v>2</v>
@@ -1784,7 +1856,13 @@
         <v>80</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA6" s="1" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="3:27" x14ac:dyDescent="0.25">
@@ -1801,7 +1879,7 @@
         <v>23</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L7" s="1">
         <v>3</v>
@@ -1827,7 +1905,13 @@
         <v>81</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="3:27" x14ac:dyDescent="0.25">
@@ -1844,7 +1928,7 @@
         <v>24</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L8" s="1">
         <v>4</v>
@@ -1872,7 +1956,7 @@
         <v>25</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L9" s="1">
         <v>5</v>
@@ -1888,7 +1972,7 @@
     </row>
     <row r="10" spans="3:27" x14ac:dyDescent="0.25">
       <c r="U10" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="V10" s="6"/>
     </row>
@@ -1902,7 +1986,7 @@
     </row>
     <row r="12" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C12" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -2083,7 +2167,7 @@
       <c r="Z16" s="6"/>
       <c r="AA16" s="6"/>
     </row>
-    <row r="17" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C17" s="1">
         <v>7</v>
       </c>
@@ -2140,7 +2224,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C18" s="1">
         <v>8</v>
       </c>
@@ -2189,13 +2273,13 @@
         <v>89</v>
       </c>
       <c r="Z18" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="AA18" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="19" spans="3:27" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C19" s="1">
         <v>9</v>
       </c>
@@ -2221,15 +2305,15 @@
         <v>92</v>
       </c>
       <c r="Z19" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="AA19" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="22" spans="3:27" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="22" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C22" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -2242,7 +2326,7 @@
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
-      <c r="O22" s="6"/>
+      <c r="O22" s="7"/>
       <c r="U22" s="6" t="s">
         <v>97</v>
       </c>
@@ -2250,7 +2334,7 @@
       <c r="W22" s="6"/>
       <c r="X22" s="6"/>
     </row>
-    <row r="23" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>0</v>
       </c>
@@ -2273,7 +2357,7 @@
         <v>60</v>
       </c>
       <c r="L23" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="M23" t="s">
         <v>61</v>
@@ -2281,9 +2365,6 @@
       <c r="N23" t="s">
         <v>62</v>
       </c>
-      <c r="O23" t="s">
-        <v>152</v>
-      </c>
       <c r="U23" t="s">
         <v>0</v>
       </c>
@@ -2297,7 +2378,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C24">
         <v>1</v>
       </c>
@@ -2320,17 +2401,15 @@
         <v>3311989</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="O24" s="1" t="s">
-        <v>151</v>
-      </c>
+      <c r="O24" s="1"/>
       <c r="U24" s="1">
         <v>1</v>
       </c>
@@ -2344,7 +2423,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="25" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C25">
         <v>2</v>
       </c>
@@ -2367,19 +2446,17 @@
         <v>331989</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="O25" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="26" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="O25" s="1"/>
+    </row>
+    <row r="26" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C26">
         <v>3</v>
       </c>
@@ -2393,7 +2470,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:28" x14ac:dyDescent="0.25">
       <c r="U27" s="6" t="s">
         <v>108</v>
       </c>
@@ -2403,7 +2480,7 @@
       <c r="Y27" s="6"/>
       <c r="Z27" s="6"/>
     </row>
-    <row r="28" spans="3:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:28" x14ac:dyDescent="0.25">
       <c r="U28" t="s">
         <v>104</v>
       </c>
@@ -2422,8 +2499,14 @@
       <c r="Z28" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="29" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="AA28" t="s">
+        <v>150</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="29" spans="3:28" x14ac:dyDescent="0.25">
       <c r="I29" s="6" t="s">
         <v>68</v>
       </c>
@@ -2433,7 +2516,7 @@
       </c>
       <c r="M29" s="6"/>
       <c r="O29" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="P29" s="6"/>
       <c r="U29" s="1">
@@ -2454,8 +2537,14 @@
       <c r="Z29" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="AA29" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AB29" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="3:28" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
         <v>0</v>
       </c>
@@ -2472,7 +2561,7 @@
         <v>0</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="U30" s="1">
         <v>6</v>
@@ -2492,8 +2581,14 @@
       <c r="Z30" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="AA30" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AB30" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="3:28" x14ac:dyDescent="0.25">
       <c r="I31" s="1">
         <v>2</v>
       </c>
@@ -2511,15 +2606,15 @@
         <v>1</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="32" spans="3:27" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="3:28" x14ac:dyDescent="0.25">
       <c r="O32" s="1">
         <v>2</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="9:27" x14ac:dyDescent="0.25">
@@ -2527,12 +2622,16 @@
         <v>3</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="U33" s="6" t="s">
         <v>109</v>
       </c>
       <c r="V33" s="6"/>
+      <c r="X33" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="Y33" s="6"/>
     </row>
     <row r="34" spans="9:27" x14ac:dyDescent="0.25">
       <c r="I34" s="6" t="s">
@@ -2549,6 +2648,12 @@
       <c r="V34" s="1" t="s">
         <v>83</v>
       </c>
+      <c r="X34" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="1" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="35" spans="9:27" x14ac:dyDescent="0.25">
       <c r="I35" t="s">
@@ -2569,6 +2674,12 @@
       <c r="V35" s="1">
         <v>3</v>
       </c>
+      <c r="X35" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="1" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="36" spans="9:27" x14ac:dyDescent="0.25">
       <c r="I36" s="1">
@@ -2587,7 +2698,7 @@
     </row>
     <row r="38" spans="9:27" x14ac:dyDescent="0.25">
       <c r="U38" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="V38" s="6"/>
       <c r="W38" s="6"/>
@@ -2598,7 +2709,7 @@
     </row>
     <row r="39" spans="9:27" x14ac:dyDescent="0.25">
       <c r="I39" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
@@ -2616,13 +2727,13 @@
         <v>83</v>
       </c>
       <c r="X39" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y39" t="s">
         <v>110</v>
       </c>
-      <c r="Y39" t="s">
-        <v>111</v>
-      </c>
       <c r="Z39" t="s">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="AA39" t="s">
         <v>10</v>
@@ -2633,19 +2744,19 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
+        <v>115</v>
+      </c>
+      <c r="K40" t="s">
+        <v>110</v>
+      </c>
+      <c r="L40" t="s">
+        <v>116</v>
+      </c>
+      <c r="M40" t="s">
         <v>117</v>
       </c>
-      <c r="K40" t="s">
-        <v>112</v>
-      </c>
-      <c r="L40" t="s">
+      <c r="N40" t="s">
         <v>118</v>
-      </c>
-      <c r="M40" t="s">
-        <v>119</v>
-      </c>
-      <c r="N40" t="s">
-        <v>120</v>
       </c>
       <c r="O40" t="s">
         <v>10</v>
@@ -2662,14 +2773,14 @@
       <c r="X40" s="4">
         <v>38718.5</v>
       </c>
-      <c r="Y40" s="4">
-        <v>38718.833333333336</v>
-      </c>
-      <c r="Z40" s="1">
-        <v>1</v>
+      <c r="Y40" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z40" s="1" t="s">
+        <v>162</v>
       </c>
       <c r="AA40" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="9:27" x14ac:dyDescent="0.25">
@@ -2686,13 +2797,13 @@
         <v>38777.5</v>
       </c>
       <c r="M41" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N41" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="O41" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="42" spans="9:27" x14ac:dyDescent="0.25">
@@ -2709,13 +2820,13 @@
         <v>38838.5</v>
       </c>
       <c r="M42" t="s">
+        <v>119</v>
+      </c>
+      <c r="N42" t="s">
+        <v>120</v>
+      </c>
+      <c r="O42" t="s">
         <v>121</v>
-      </c>
-      <c r="N42" t="s">
-        <v>122</v>
-      </c>
-      <c r="O42" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="43" spans="9:27" x14ac:dyDescent="0.25">
@@ -2732,16 +2843,16 @@
         <v>38718.875</v>
       </c>
       <c r="M43" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="N43" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="O43" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="U43" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
@@ -2764,13 +2875,13 @@
         <v>38838.541666666664</v>
       </c>
       <c r="M44" t="s">
+        <v>122</v>
+      </c>
+      <c r="N44" t="s">
         <v>124</v>
       </c>
-      <c r="N44" t="s">
-        <v>126</v>
-      </c>
       <c r="O44" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="U44" t="s">
         <v>0</v>
@@ -2782,13 +2893,13 @@
         <v>83</v>
       </c>
       <c r="X44" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y44" t="s">
         <v>110</v>
       </c>
-      <c r="Y44" t="s">
-        <v>111</v>
-      </c>
       <c r="Z44" t="s">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="AA44" t="s">
         <v>10</v>
@@ -2807,24 +2918,24 @@
       <c r="X45" s="4">
         <v>38838.5</v>
       </c>
-      <c r="Y45" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="Z45" s="1">
-        <v>1</v>
+      <c r="Y45" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z45" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="AA45" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="9:27" x14ac:dyDescent="0.25">
       <c r="I47" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J47" s="6"/>
       <c r="K47" s="6"/>
       <c r="M47" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="N47" s="6"/>
       <c r="O47" s="6"/>
@@ -2834,19 +2945,19 @@
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K48" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="M48" t="s">
         <v>0</v>
       </c>
       <c r="N48" t="s">
+        <v>134</v>
+      </c>
+      <c r="O48" t="s">
         <v>136</v>
-      </c>
-      <c r="O48" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="49" spans="9:15" x14ac:dyDescent="0.25">
@@ -2871,7 +2982,7 @@
     </row>
     <row r="52" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I52" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J52" s="6"/>
       <c r="K52" s="6"/>
@@ -2887,13 +2998,13 @@
         <v>59</v>
       </c>
       <c r="K53" t="s">
+        <v>116</v>
+      </c>
+      <c r="L53" t="s">
+        <v>117</v>
+      </c>
+      <c r="M53" t="s">
         <v>118</v>
-      </c>
-      <c r="L53" t="s">
-        <v>119</v>
-      </c>
-      <c r="M53" t="s">
-        <v>120</v>
       </c>
       <c r="N53" t="s">
         <v>10</v>
@@ -2910,13 +3021,13 @@
         <v>39203.5</v>
       </c>
       <c r="L54" t="s">
+        <v>138</v>
+      </c>
+      <c r="M54" t="s">
+        <v>139</v>
+      </c>
+      <c r="N54" t="s">
         <v>140</v>
-      </c>
-      <c r="M54" t="s">
-        <v>141</v>
-      </c>
-      <c r="N54" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="55" spans="9:15" x14ac:dyDescent="0.25">
@@ -2930,18 +3041,18 @@
         <v>38869.5</v>
       </c>
       <c r="L55" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="M55" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="N55" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I58" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="6"/>
@@ -2953,16 +3064,16 @@
         <v>0</v>
       </c>
       <c r="J59" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K59" t="s">
         <v>107</v>
       </c>
       <c r="L59" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="M59" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" spans="9:15" ht="30" x14ac:dyDescent="0.25">
@@ -2976,14 +3087,31 @@
         <v>1</v>
       </c>
       <c r="L60" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="M60" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="25">
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="M47:O47"/>
+    <mergeCell ref="I52:N52"/>
+    <mergeCell ref="I58:M58"/>
+    <mergeCell ref="U33:V33"/>
+    <mergeCell ref="U38:AA38"/>
+    <mergeCell ref="U43:AA43"/>
+    <mergeCell ref="I39:O39"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="X33:Y33"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="U16:AA16"/>
+    <mergeCell ref="I22:N22"/>
     <mergeCell ref="U3:Y3"/>
     <mergeCell ref="U22:X22"/>
     <mergeCell ref="I29:J29"/>
@@ -2992,26 +3120,11 @@
     <mergeCell ref="U27:Z27"/>
     <mergeCell ref="I3:R3"/>
     <mergeCell ref="I12:Q12"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="I22:O22"/>
-    <mergeCell ref="U16:AA16"/>
-    <mergeCell ref="U38:AA38"/>
-    <mergeCell ref="U43:AA43"/>
-    <mergeCell ref="I39:O39"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="M47:O47"/>
-    <mergeCell ref="I52:N52"/>
-    <mergeCell ref="I58:M58"/>
-    <mergeCell ref="U33:V33"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="24">
+  <tableParts count="25">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
@@ -3036,6 +3149,7 @@
     <tablePart r:id="rId23"/>
     <tablePart r:id="rId24"/>
     <tablePart r:id="rId25"/>
+    <tablePart r:id="rId26"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>